<commit_message>
DSG gen working and fix Ranalysis
</commit_message>
<xml_diff>
--- a/test/resources/dsg/DSG-STD-test.xlsx
+++ b/test/resources/dsg/DSG-STD-test.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaell\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaell\Desktop\Project\hascoapi\test\resources\dsg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DF52CE3-56DD-434C-A468-508F910A41FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C6BCDE4-A0DF-481E-BA90-65BA4E054CEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="5652" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="InfoSheet" sheetId="1" r:id="rId1"/>
-    <sheet name="Namespaces" sheetId="2" r:id="rId2"/>
+    <sheet name="Namespace" sheetId="2" r:id="rId2"/>
     <sheet name="SSD" sheetId="3" r:id="rId3"/>
     <sheet name="STD" sheetId="4" r:id="rId4"/>
     <sheet name="VD" sheetId="5" r:id="rId5"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="940" uniqueCount="610">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="949" uniqueCount="613">
   <si>
     <t>hasStudyURI</t>
   </si>
@@ -1860,6 +1860,15 @@
   </si>
   <si>
     <t>??response-optioncollection</t>
+  </si>
+  <si>
+    <t>hasScope</t>
+  </si>
+  <si>
+    <t>groundingLabel</t>
+  </si>
+  <si>
+    <t>role</t>
   </si>
 </sst>
 </file>
@@ -2877,7 +2886,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.5703125" customWidth="1"/>
@@ -2887,7 +2896,7 @@
     <col min="5" max="5" width="21.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>24</v>
       </c>
@@ -2910,13 +2919,22 @@
         <v>30</v>
       </c>
       <c r="H1" t="s">
+        <v>612</v>
+      </c>
+      <c r="I1" t="s">
+        <v>611</v>
+      </c>
+      <c r="J1" t="s">
+        <v>610</v>
+      </c>
+      <c r="K1" t="s">
+        <v>32</v>
+      </c>
+      <c r="L1" t="s">
         <v>31</v>
       </c>
-      <c r="I1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>562</v>
       </c>
@@ -2935,8 +2953,11 @@
       <c r="F2" t="s">
         <v>570</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J2" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>563</v>
       </c>
@@ -2955,8 +2976,11 @@
       <c r="F3" t="s">
         <v>571</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J3" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>564</v>
       </c>
@@ -2975,8 +2999,11 @@
       <c r="F4" t="s">
         <v>572</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J4" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>565</v>
       </c>
@@ -2995,8 +3022,11 @@
       <c r="F5" t="s">
         <v>573</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J5" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>566</v>
       </c>
@@ -3015,8 +3045,11 @@
       <c r="F6" t="s">
         <v>574</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J6" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>567</v>
       </c>
@@ -3034,6 +3067,9 @@
       </c>
       <c r="F7" t="s">
         <v>575</v>
+      </c>
+      <c r="J7" t="s">
+        <v>599</v>
       </c>
     </row>
   </sheetData>

</xml_diff>